<commit_message>
merged-cells-ext: tested and fixed accumulating and appending of 'merged' range type
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Range_Merged.xlsx
+++ b/Ref_Files/Test_Range_Merged.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="10">
   <si>
     <t xml:space="preserve">Операция Х-00100, с два реда</t>
   </si>
@@ -64,6 +64,15 @@
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00203 измерване</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Операция Х-00300, с два реда</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      -  операция Х-00301 измерване</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      -  операция Х-00302 измерване</t>
   </si>
 </sst>
 </file>
@@ -379,7 +388,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M1048576"/>
+  <dimension ref="A1:XFD1048576"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
@@ -434,9 +443,6 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="0"/>
-      <c r="L3" s="0"/>
-      <c r="M3" s="0"/>
     </row>
     <row r="4" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
@@ -455,9 +461,6 @@
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="0"/>
-      <c r="L4" s="0"/>
-      <c r="M4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
@@ -528,9 +531,6 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
-      <c r="K9" s="0"/>
-      <c r="L9" s="0"/>
-      <c r="M9" s="0"/>
     </row>
     <row r="10" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2"/>
@@ -549,9 +549,6 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
-      <c r="K10" s="0"/>
-      <c r="L10" s="0"/>
-      <c r="M10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
@@ -607,6 +604,202 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
     </row>
+    <row r="15" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="XEL15" s="0"/>
+      <c r="XEM15" s="0"/>
+      <c r="XEN15" s="0"/>
+      <c r="XEO15" s="0"/>
+      <c r="XEP15" s="0"/>
+      <c r="XEQ15" s="0"/>
+      <c r="XER15" s="0"/>
+      <c r="XES15" s="0"/>
+      <c r="XET15" s="0"/>
+      <c r="XEU15" s="0"/>
+      <c r="XEV15" s="0"/>
+      <c r="XEW15" s="0"/>
+      <c r="XEX15" s="0"/>
+      <c r="XEY15" s="0"/>
+      <c r="XEZ15" s="0"/>
+      <c r="XFA15" s="0"/>
+      <c r="XFB15" s="0"/>
+      <c r="XFC15" s="0"/>
+      <c r="XFD15" s="0"/>
+    </row>
+    <row r="16" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2"/>
+      <c r="B16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="XEL16" s="0"/>
+      <c r="XEM16" s="0"/>
+      <c r="XEN16" s="0"/>
+      <c r="XEO16" s="0"/>
+      <c r="XEP16" s="0"/>
+      <c r="XEQ16" s="0"/>
+      <c r="XER16" s="0"/>
+      <c r="XES16" s="0"/>
+      <c r="XET16" s="0"/>
+      <c r="XEU16" s="0"/>
+      <c r="XEV16" s="0"/>
+      <c r="XEW16" s="0"/>
+      <c r="XEX16" s="0"/>
+      <c r="XEY16" s="0"/>
+      <c r="XEZ16" s="0"/>
+      <c r="XFA16" s="0"/>
+      <c r="XFB16" s="0"/>
+      <c r="XFC16" s="0"/>
+      <c r="XFD16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2"/>
+      <c r="B17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="XEL17" s="0"/>
+      <c r="XEM17" s="0"/>
+      <c r="XEN17" s="0"/>
+      <c r="XEO17" s="0"/>
+      <c r="XEP17" s="0"/>
+      <c r="XEQ17" s="0"/>
+      <c r="XER17" s="0"/>
+      <c r="XES17" s="0"/>
+      <c r="XET17" s="0"/>
+      <c r="XEU17" s="0"/>
+      <c r="XEV17" s="0"/>
+      <c r="XEW17" s="0"/>
+      <c r="XEX17" s="0"/>
+      <c r="XEY17" s="0"/>
+      <c r="XEZ17" s="0"/>
+      <c r="XFA17" s="0"/>
+      <c r="XFB17" s="0"/>
+      <c r="XFC17" s="0"/>
+      <c r="XFD17" s="0"/>
+    </row>
+    <row r="18" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2"/>
+      <c r="B20" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2"/>
+      <c r="B21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2"/>
+      <c r="B23" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+    </row>
+    <row r="1048521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -661,12 +854,15 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="A9:A12"/>
     <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A23"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
merged-cells-ext: extended test to verify wrong order handling
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Range_Merged.xlsx
+++ b/Ref_Files/Test_Range_Merged.xlsx
@@ -54,7 +54,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Операция Х-00200, с три реда</t>
+    <t xml:space="preserve">Операция Х-00200, с четири реда</t>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00201 измерване</t>
@@ -66,7 +66,7 @@
     <t xml:space="preserve">      -  операция Х-00203 измерване</t>
   </si>
   <si>
-    <t xml:space="preserve">Операция Х-00300, с два реда</t>
+    <t xml:space="preserve">Операция Х-00300, с три реда</t>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00301 измерване</t>
@@ -619,25 +619,6 @@
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
-      <c r="XEL15" s="0"/>
-      <c r="XEM15" s="0"/>
-      <c r="XEN15" s="0"/>
-      <c r="XEO15" s="0"/>
-      <c r="XEP15" s="0"/>
-      <c r="XEQ15" s="0"/>
-      <c r="XER15" s="0"/>
-      <c r="XES15" s="0"/>
-      <c r="XET15" s="0"/>
-      <c r="XEU15" s="0"/>
-      <c r="XEV15" s="0"/>
-      <c r="XEW15" s="0"/>
-      <c r="XEX15" s="0"/>
-      <c r="XEY15" s="0"/>
-      <c r="XEZ15" s="0"/>
-      <c r="XFA15" s="0"/>
-      <c r="XFB15" s="0"/>
-      <c r="XFC15" s="0"/>
-      <c r="XFD15" s="0"/>
     </row>
     <row r="16" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -656,25 +637,6 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
-      <c r="XEL16" s="0"/>
-      <c r="XEM16" s="0"/>
-      <c r="XEN16" s="0"/>
-      <c r="XEO16" s="0"/>
-      <c r="XEP16" s="0"/>
-      <c r="XEQ16" s="0"/>
-      <c r="XER16" s="0"/>
-      <c r="XES16" s="0"/>
-      <c r="XET16" s="0"/>
-      <c r="XEU16" s="0"/>
-      <c r="XEV16" s="0"/>
-      <c r="XEW16" s="0"/>
-      <c r="XEX16" s="0"/>
-      <c r="XEY16" s="0"/>
-      <c r="XEZ16" s="0"/>
-      <c r="XFA16" s="0"/>
-      <c r="XFB16" s="0"/>
-      <c r="XFC16" s="0"/>
-      <c r="XFD16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
@@ -689,25 +651,25 @@
       </c>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-      <c r="XEL17" s="0"/>
-      <c r="XEM17" s="0"/>
-      <c r="XEN17" s="0"/>
-      <c r="XEO17" s="0"/>
-      <c r="XEP17" s="0"/>
-      <c r="XEQ17" s="0"/>
-      <c r="XER17" s="0"/>
-      <c r="XES17" s="0"/>
-      <c r="XET17" s="0"/>
-      <c r="XEU17" s="0"/>
-      <c r="XEV17" s="0"/>
-      <c r="XEW17" s="0"/>
-      <c r="XEX17" s="0"/>
-      <c r="XEY17" s="0"/>
-      <c r="XEZ17" s="0"/>
-      <c r="XFA17" s="0"/>
-      <c r="XFB17" s="0"/>
-      <c r="XFC17" s="0"/>
-      <c r="XFD17" s="0"/>
+      <c r="XEL17" s="6"/>
+      <c r="XEM17" s="6"/>
+      <c r="XEN17" s="6"/>
+      <c r="XEO17" s="6"/>
+      <c r="XEP17" s="6"/>
+      <c r="XEQ17" s="6"/>
+      <c r="XER17" s="6"/>
+      <c r="XES17" s="6"/>
+      <c r="XET17" s="6"/>
+      <c r="XEU17" s="6"/>
+      <c r="XEV17" s="6"/>
+      <c r="XEW17" s="6"/>
+      <c r="XEX17" s="6"/>
+      <c r="XEY17" s="6"/>
+      <c r="XEZ17" s="6"/>
+      <c r="XFA17" s="6"/>
+      <c r="XFB17" s="6"/>
+      <c r="XFC17" s="6"/>
+      <c r="XFD17" s="6"/>
     </row>
     <row r="18" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="n">
@@ -728,13 +690,13 @@
     <row r="19" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
       <c r="B19" s="5" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
@@ -752,7 +714,7 @@
         <v>2</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -760,13 +722,13 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
       <c r="B21" s="5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>

</xml_diff>

<commit_message>
merged-cells-ext: extended test file to support larger section
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Range_Merged.xlsx
+++ b/Ref_Files/Test_Range_Merged.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="11">
   <si>
     <t xml:space="preserve">Операция Х-00100, с два реда</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00203 измерване</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      -  операция Х-99999 измерване</t>
   </si>
   <si>
     <t xml:space="preserve">Операция Х-00300, с три реда</t>
@@ -604,33 +607,48 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2"/>
+      <c r="B15" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
+      <c r="C15" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>999</v>
+      </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
+      <c r="XEL15" s="0"/>
+      <c r="XEM15" s="0"/>
+      <c r="XEN15" s="0"/>
+      <c r="XEO15" s="0"/>
+      <c r="XEP15" s="0"/>
+      <c r="XEQ15" s="0"/>
+      <c r="XER15" s="0"/>
+      <c r="XES15" s="0"/>
+      <c r="XET15" s="0"/>
+      <c r="XEU15" s="0"/>
+      <c r="XEV15" s="0"/>
+      <c r="XEW15" s="0"/>
+      <c r="XEX15" s="0"/>
+      <c r="XEY15" s="0"/>
+      <c r="XEZ15" s="0"/>
+      <c r="XFA15" s="0"/>
+      <c r="XFB15" s="0"/>
+      <c r="XFC15" s="0"/>
+      <c r="XFD15" s="0"/>
     </row>
     <row r="16" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>100</v>
-      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="1"/>
@@ -638,7 +656,7 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
       <c r="B17" s="5" t="s">
         <v>9</v>
@@ -651,53 +669,53 @@
       </c>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-      <c r="XEL17" s="6"/>
-      <c r="XEM17" s="6"/>
-      <c r="XEN17" s="6"/>
-      <c r="XEO17" s="6"/>
-      <c r="XEP17" s="6"/>
-      <c r="XEQ17" s="6"/>
-      <c r="XER17" s="6"/>
-      <c r="XES17" s="6"/>
-      <c r="XET17" s="6"/>
-      <c r="XEU17" s="6"/>
-      <c r="XEV17" s="6"/>
-      <c r="XEW17" s="6"/>
-      <c r="XEX17" s="6"/>
-      <c r="XEY17" s="6"/>
-      <c r="XEZ17" s="6"/>
-      <c r="XFA17" s="6"/>
-      <c r="XFB17" s="6"/>
-      <c r="XFC17" s="6"/>
-      <c r="XFD17" s="6"/>
-    </row>
-    <row r="18" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2"/>
+      <c r="B18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
+      <c r="XEL18" s="6"/>
+      <c r="XEM18" s="6"/>
+      <c r="XEN18" s="6"/>
+      <c r="XEO18" s="6"/>
+      <c r="XEP18" s="6"/>
+      <c r="XEQ18" s="6"/>
+      <c r="XER18" s="6"/>
+      <c r="XES18" s="6"/>
+      <c r="XET18" s="6"/>
+      <c r="XEU18" s="6"/>
+      <c r="XEV18" s="6"/>
+      <c r="XEW18" s="6"/>
+      <c r="XEX18" s="6"/>
+      <c r="XEY18" s="6"/>
+      <c r="XEZ18" s="6"/>
+      <c r="XFA18" s="6"/>
+      <c r="XFB18" s="6"/>
+      <c r="XFC18" s="6"/>
+      <c r="XFD18" s="6"/>
     </row>
     <row r="19" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-      <c r="B19" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>5</v>
-      </c>
+      <c r="A19" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="1"/>
@@ -705,61 +723,78 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
       <c r="B20" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
       <c r="B21" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
+      <c r="A22" s="2"/>
+      <c r="B22" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>7</v>
+      </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
-      <c r="B23" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>100</v>
-      </c>
+      <c r="A23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
-    <row r="1048521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2"/>
+      <c r="B24" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+    </row>
     <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -821,10 +856,10 @@
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A23:A24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
merged-cells-ext: incomplete implementation - keep version
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Range_Merged.xlsx
+++ b/Ref_Files/Test_Range_Merged.xlsx
@@ -1,34 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr filterPrivacy="1"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView activeTab="0" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="КСС_ОП1" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="Prices" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">#REF!</definedName>
+    <definedName name="_Hlk165973344" localSheetId="0" hidden="0">#REF!</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="11">
   <si>
-    <t xml:space="preserve">Операция Х-00100, с два реда</t>
+    <t>Операция Х-00100, с два реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00100 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <r>
@@ -39,7 +37,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">m</t>
+      <t>m</t>
     </r>
     <r>
       <rPr>
@@ -50,42 +48,51 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">3</t>
+      <t>3</t>
     </r>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">Операция Х-00200, с четири реда</t>
+    <t>Операция Х-00200, с четири реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00201 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00202 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00203 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-99999 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">Операция Х-00300, с три реда</t>
+    <t>Операция Х-00300, с три реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00301 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00302 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,14 +140,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
@@ -149,58 +156,58 @@
     </border>
   </borders>
   <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -211,11 +218,17 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Тема на Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема на Office">
   <a:themeElements>
     <a:clrScheme name="Оffice">
       <a:dk1>
@@ -257,12 +270,12 @@
     </a:clrScheme>
     <a:fontScheme name="Оffice">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -294,7 +307,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -318,7 +331,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -378,38 +391,37 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:XFD24"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" outlineLevelCol="0" outlineLevelRow="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.84"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="7" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16365" min="14" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16366" style="1" width="10.16"/>
+    <col min="1" max="1" width="10.14" customWidth="1" style="1"/>
+    <col min="2" max="2" width="38.47" customWidth="1" style="1"/>
+    <col min="3" max="3" width="10.7" customWidth="1" style="1"/>
+    <col min="4" max="4" width="7.86" customWidth="1" style="1"/>
+    <col min="5" max="5" width="7.35" customWidth="1" style="1"/>
+    <col min="6" max="6" width="7.84" customWidth="1" style="1"/>
+    <col min="7" max="10" width="9.14" customWidth="1" style="1"/>
+    <col min="14" max="16365" width="9.14" customWidth="1" style="1"/>
+    <col min="16366" max="16384" width="10.16" customWidth="1" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="n">
+    <row r="1" spans="1:6" ht="15">
+      <c r="A1" s="2">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C1" s="4"/>
@@ -417,25 +429,25 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:6" ht="15">
       <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4" t="n">
+      <c r="C2" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
         <v>100</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
     </row>
-    <row r="3" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="3" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C3" s="4"/>
@@ -447,15 +459,15 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A4" s="2"/>
-      <c r="B4" s="5" t="s">
+      <c r="B4" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="C4" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
         <v>100</v>
       </c>
       <c r="E4" s="4"/>
@@ -465,39 +477,39 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:6" ht="15">
       <c r="A5" s="2"/>
-      <c r="B5" s="5" t="s">
+      <c r="B5" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="C5" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
         <v>100</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:6" ht="15">
       <c r="A6" s="2"/>
-      <c r="B6" s="5" t="s">
+      <c r="B6" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="C6" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4">
         <v>100</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" spans="1:6" ht="15">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C7" s="4"/>
@@ -505,25 +517,25 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:6" ht="15">
       <c r="A8" s="2"/>
-      <c r="B8" s="5" t="s">
+      <c r="B8" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="C8" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
         <v>100</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+    <row r="9" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A9" s="2">
         <v>4</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C9" s="4"/>
@@ -535,15 +547,15 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="C10" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D10" s="4">
         <v>100</v>
       </c>
       <c r="E10" s="4"/>
@@ -553,39 +565,39 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:6" ht="15">
       <c r="A11" s="2"/>
-      <c r="B11" s="5" t="s">
+      <c r="B11" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="4" t="n">
+      <c r="C11" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
         <v>100</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:6" ht="15">
       <c r="A12" s="2"/>
-      <c r="B12" s="5" t="s">
+      <c r="B12" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D12" s="4" t="n">
+      <c r="C12" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
         <v>100</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+    <row r="13" spans="1:6" ht="15">
+      <c r="A13" s="2">
         <v>5</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C13" s="4"/>
@@ -593,58 +605,58 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:6" ht="15">
       <c r="A14" s="2"/>
-      <c r="B14" s="5" t="s">
+      <c r="B14" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="4" t="n">
+      <c r="C14" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4">
         <v>100</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:16384" ht="15">
       <c r="A15" s="2"/>
-      <c r="B15" s="5" t="s">
+      <c r="B15" t="s" s="5">
         <v>7</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D15" s="4" t="n">
+      <c r="C15" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4">
         <v>999</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="XEL15" s="0"/>
-      <c r="XEM15" s="0"/>
-      <c r="XEN15" s="0"/>
-      <c r="XEO15" s="0"/>
-      <c r="XEP15" s="0"/>
-      <c r="XEQ15" s="0"/>
-      <c r="XER15" s="0"/>
-      <c r="XES15" s="0"/>
-      <c r="XET15" s="0"/>
-      <c r="XEU15" s="0"/>
-      <c r="XEV15" s="0"/>
-      <c r="XEW15" s="0"/>
-      <c r="XEX15" s="0"/>
-      <c r="XEY15" s="0"/>
-      <c r="XEZ15" s="0"/>
-      <c r="XFA15" s="0"/>
-      <c r="XFB15" s="0"/>
-      <c r="XFC15" s="0"/>
-      <c r="XFD15" s="0"/>
-    </row>
-    <row r="16" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
+      <c r="XEL15"/>
+      <c r="XEM15"/>
+      <c r="XEN15"/>
+      <c r="XEO15"/>
+      <c r="XEP15"/>
+      <c r="XEQ15"/>
+      <c r="XER15"/>
+      <c r="XES15"/>
+      <c r="XET15"/>
+      <c r="XEU15"/>
+      <c r="XEV15"/>
+      <c r="XEW15"/>
+      <c r="XEX15"/>
+      <c r="XEY15"/>
+      <c r="XEZ15"/>
+      <c r="XFA15"/>
+      <c r="XFB15"/>
+      <c r="XFC15"/>
+      <c r="XFD15"/>
+    </row>
+    <row r="16" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A16" s="2">
         <v>6</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" t="s" s="3">
         <v>8</v>
       </c>
       <c r="C16" s="4"/>
@@ -656,15 +668,15 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A17" s="2"/>
-      <c r="B17" s="5" t="s">
+      <c r="B17" t="s" s="5">
         <v>9</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D17" s="4" t="n">
+      <c r="C17" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D17" s="4">
         <v>100</v>
       </c>
       <c r="E17" s="4"/>
@@ -674,15 +686,15 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:16384" ht="15">
       <c r="A18" s="2"/>
-      <c r="B18" s="5" t="s">
+      <c r="B18" t="s" s="5">
         <v>10</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="4" t="n">
+      <c r="C18" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D18" s="4">
         <v>100</v>
       </c>
       <c r="E18" s="4"/>
@@ -707,11 +719,11 @@
       <c r="XFC18" s="6"/>
       <c r="XFD18" s="6"/>
     </row>
-    <row r="19" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="n">
+    <row r="19" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A19" s="2">
         <v>7</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C19" s="4"/>
@@ -723,15 +735,15 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A20" s="2"/>
-      <c r="B20" s="5" t="s">
+      <c r="B20" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="4" t="n">
+      <c r="C20" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4">
         <v>5</v>
       </c>
       <c r="E20" s="4"/>
@@ -741,39 +753,39 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:6" ht="15">
       <c r="A21" s="2"/>
-      <c r="B21" s="5" t="s">
+      <c r="B21" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" s="4" t="n">
+      <c r="C21" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4">
         <v>6</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:6" ht="15">
       <c r="A22" s="2"/>
-      <c r="B22" s="5" t="s">
+      <c r="B22" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D22" s="4" t="n">
+      <c r="C22" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D22" s="4">
         <v>7</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="n">
+    <row r="23" spans="1:6" ht="15">
+      <c r="A23" s="2">
         <v>8</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C23" s="4"/>
@@ -781,75 +793,75 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:6" ht="15">
       <c r="A24" s="2"/>
-      <c r="B24" s="5" t="s">
+      <c r="B24" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" s="4" t="n">
+      <c r="C24" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D24" s="4">
         <v>100</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" ht="12.8"/>
+    <row r="1048523" ht="12.8"/>
+    <row r="1048524" ht="12.8"/>
+    <row r="1048525" ht="12.8"/>
+    <row r="1048526" ht="12.8"/>
+    <row r="1048527" ht="12.8"/>
+    <row r="1048528" ht="12.8"/>
+    <row r="1048529" ht="12.8"/>
+    <row r="1048530" ht="12.8"/>
+    <row r="1048531" ht="12.8"/>
+    <row r="1048532" ht="12.8"/>
+    <row r="1048533" ht="12.8"/>
+    <row r="1048534" ht="12.8"/>
+    <row r="1048535" ht="12.8"/>
+    <row r="1048536" ht="12.8"/>
+    <row r="1048537" ht="12.8"/>
+    <row r="1048538" ht="12.8"/>
+    <row r="1048539" ht="12.8"/>
+    <row r="1048540" ht="12.8"/>
+    <row r="1048541" ht="12.8"/>
+    <row r="1048542" ht="12.8"/>
+    <row r="1048543" ht="12.8"/>
+    <row r="1048544" ht="12.8"/>
+    <row r="1048545" ht="12.8"/>
+    <row r="1048546" ht="12.8"/>
+    <row r="1048547" ht="12.8"/>
+    <row r="1048548" ht="12.8"/>
+    <row r="1048549" ht="12.8"/>
+    <row r="1048550" ht="12.8"/>
+    <row r="1048551" ht="12.8"/>
+    <row r="1048552" ht="12.8"/>
+    <row r="1048553" ht="12.8"/>
+    <row r="1048554" ht="12.8"/>
+    <row r="1048555" ht="12.8"/>
+    <row r="1048556" ht="12.8"/>
+    <row r="1048557" ht="12.8"/>
+    <row r="1048558" ht="12.8"/>
+    <row r="1048559" ht="12.8"/>
+    <row r="1048560" ht="12.8"/>
+    <row r="1048561" ht="12.8"/>
+    <row r="1048562" ht="12.8"/>
+    <row r="1048563" ht="12.8"/>
+    <row r="1048564" ht="12.8"/>
+    <row r="1048565" ht="12.8"/>
+    <row r="1048566" ht="12.8"/>
+    <row r="1048567" ht="12.8"/>
+    <row r="1048568" ht="12.8"/>
+    <row r="1048569" ht="12.8"/>
+    <row r="1048570" ht="12.8"/>
+    <row r="1048571" ht="12.8"/>
+    <row r="1048572" ht="12.8"/>
+    <row r="1048573" ht="12.8"/>
+    <row r="1048574" ht="12.8"/>
+    <row r="1048575" ht="12.8"/>
+    <row r="1048576" ht="12.8"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:A2"/>
@@ -861,12 +873,207 @@
     <mergeCell ref="A19:A22"/>
     <mergeCell ref="A23:A24"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <phoneticPr fontId="1"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" scale="100" orientation="portrait" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr/>
+  <cols>
+    <col min="1" max="1" width="10.14" customWidth="1"/>
+    <col min="2" max="2" width="38.47" customWidth="1"/>
+    <col min="3" max="3" width="10.7" customWidth="1"/>
+    <col min="4" max="4" width="7.86" customWidth="1"/>
+    <col min="5" max="5" width="7.35" customWidth="1"/>
+    <col min="6" max="6" width="7.84" customWidth="1"/>
+    <col min="7" max="9" width="9.14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15" customHeight="1">
+      <c r="A1" s="2">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s" s="3">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1">
+      <c r="A2" s="2"/>
+      <c r="B2" t="s" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
+        <v>300</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" customHeight="1">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="3">
+        <v>3</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" ht="15" customHeight="1">
+      <c r="A4" s="2"/>
+      <c r="B4" t="s" s="5">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
+        <v>207</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1">
+      <c r="A5" s="2"/>
+      <c r="B5" t="s" s="5">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
+        <v>206</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:6" ht="15" customHeight="1">
+      <c r="A6" s="2"/>
+      <c r="B6" t="s" s="5">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4">
+        <v>205</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s" s="3">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1">
+      <c r="A8" s="2"/>
+      <c r="B8" t="s" s="5">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
+        <v>100</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1">
+      <c r="A9" s="2"/>
+      <c r="B9" t="s" s="5">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4">
+        <v>999</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" ht="15" customHeight="1">
+      <c r="A10" s="2">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s" s="3">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" ht="15" customHeight="1">
+      <c r="A11" s="2"/>
+      <c r="B11" t="s" s="5">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
+        <v>100</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1">
+      <c r="A12" s="2"/>
+      <c r="B12" t="s" s="5">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
+        <v>100</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:A12"/>
+  </mergeCells>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
merged-cells-ext: can locate all rows, which belong to a group, but must apply merging of cells, when needed
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Range_Merged.xlsx
+++ b/Ref_Files/Test_Range_Merged.xlsx
@@ -1,34 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr filterPrivacy="1"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView activeTab="0" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="КСС_ОП1" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="Prices" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">#REF!</definedName>
+    <definedName name="_Hlk165973344" localSheetId="0" hidden="0">#REF!</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="13">
   <si>
-    <t xml:space="preserve">Операция Х-00100, с два реда</t>
+    <t>Операция Х-00100, с два реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00100 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <r>
@@ -39,7 +37,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">m</t>
+      <t>m</t>
     </r>
     <r>
       <rPr>
@@ -50,48 +48,59 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">3</t>
+      <t>3</t>
     </r>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">Операция Х-00200, с четири реда</t>
+    <t>Операция Х-00200, с четири реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00201 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00202 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00203 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-99999 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">Операция Х-00300, с три реда</t>
+    <t>Операция Х-00300, с три реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00301 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00302 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-88888 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-77777 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,14 +148,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
@@ -155,58 +164,58 @@
     </border>
   </borders>
   <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -217,11 +226,17 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Тема на Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема на Office">
   <a:themeElements>
     <a:clrScheme name="Оffice">
       <a:dk1>
@@ -263,12 +278,12 @@
     </a:clrScheme>
     <a:fontScheme name="Оffice">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -300,7 +315,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -324,7 +339,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -384,38 +399,37 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:XFD29"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" outlineLevelCol="0" outlineLevelRow="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.84"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="7" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16365" min="14" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16366" style="1" width="10.16"/>
+    <col min="1" max="1" width="10.14" customWidth="1" style="1"/>
+    <col min="2" max="2" width="38.47" customWidth="1" style="1"/>
+    <col min="3" max="3" width="10.7" customWidth="1" style="1"/>
+    <col min="4" max="4" width="7.86" customWidth="1" style="1"/>
+    <col min="5" max="5" width="7.35" customWidth="1" style="1"/>
+    <col min="6" max="6" width="7.84" customWidth="1" style="1"/>
+    <col min="7" max="10" width="9.14" customWidth="1" style="1"/>
+    <col min="14" max="16365" width="9.14" customWidth="1" style="1"/>
+    <col min="16366" max="16384" width="10.16" customWidth="1" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="n">
+    <row r="1" spans="1:6" ht="15">
+      <c r="A1" s="2">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C1" s="4"/>
@@ -423,25 +437,25 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:6" ht="15">
       <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4" t="n">
+      <c r="C2" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
         <v>100</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
     </row>
-    <row r="3" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="3" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C3" s="4"/>
@@ -453,15 +467,15 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A4" s="2"/>
-      <c r="B4" s="5" t="s">
+      <c r="B4" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="C4" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
         <v>100</v>
       </c>
       <c r="E4" s="4"/>
@@ -471,39 +485,39 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:6" ht="15">
       <c r="A5" s="2"/>
-      <c r="B5" s="5" t="s">
+      <c r="B5" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="C5" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
         <v>100</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:6" ht="15">
       <c r="A6" s="2"/>
-      <c r="B6" s="5" t="s">
+      <c r="B6" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="C6" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4">
         <v>100</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" spans="1:6" ht="15">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C7" s="4"/>
@@ -511,25 +525,25 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:6" ht="15">
       <c r="A8" s="2"/>
-      <c r="B8" s="5" t="s">
+      <c r="B8" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="C8" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
         <v>100</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+    <row r="9" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A9" s="2">
         <v>4</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C9" s="4"/>
@@ -541,15 +555,15 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="C10" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D10" s="4">
         <v>100</v>
       </c>
       <c r="E10" s="4"/>
@@ -559,39 +573,39 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:6" ht="15">
       <c r="A11" s="2"/>
-      <c r="B11" s="5" t="s">
+      <c r="B11" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="4" t="n">
+      <c r="C11" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
         <v>100</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:6" ht="15">
       <c r="A12" s="2"/>
-      <c r="B12" s="5" t="s">
+      <c r="B12" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D12" s="4" t="n">
+      <c r="C12" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
         <v>100</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+    <row r="13" spans="1:6" ht="15">
+      <c r="A13" s="2">
         <v>5</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C13" s="4"/>
@@ -599,39 +613,39 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:6" ht="15">
       <c r="A14" s="2"/>
-      <c r="B14" s="5" t="s">
+      <c r="B14" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="4" t="n">
+      <c r="C14" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4">
         <v>100</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:6" ht="15">
       <c r="A15" s="2"/>
-      <c r="B15" s="5" t="s">
+      <c r="B15" t="s" s="5">
         <v>7</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D15" s="4" t="n">
+      <c r="C15" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4">
         <v>999</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
+    <row r="16" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A16" s="2">
         <v>6</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" t="s" s="3">
         <v>8</v>
       </c>
       <c r="C16" s="4"/>
@@ -643,15 +657,15 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A17" s="2"/>
-      <c r="B17" s="5" t="s">
+      <c r="B17" t="s" s="5">
         <v>9</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D17" s="4" t="n">
+      <c r="C17" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D17" s="4">
         <v>100</v>
       </c>
       <c r="E17" s="4"/>
@@ -661,15 +675,15 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:16384" ht="15">
       <c r="A18" s="2"/>
-      <c r="B18" s="5" t="s">
+      <c r="B18" t="s" s="5">
         <v>10</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="4" t="n">
+      <c r="C18" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D18" s="4">
         <v>100</v>
       </c>
       <c r="E18" s="4"/>
@@ -694,11 +708,11 @@
       <c r="XFC18" s="6"/>
       <c r="XFD18" s="6"/>
     </row>
-    <row r="19" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="n">
+    <row r="19" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A19" s="2">
         <v>7</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C19" s="4"/>
@@ -710,15 +724,15 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A20" s="2"/>
-      <c r="B20" s="5" t="s">
+      <c r="B20" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="4" t="n">
+      <c r="C20" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4">
         <v>5</v>
       </c>
       <c r="E20" s="4"/>
@@ -728,39 +742,39 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:6" ht="15">
       <c r="A21" s="2"/>
-      <c r="B21" s="5" t="s">
+      <c r="B21" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" s="4" t="n">
+      <c r="C21" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4">
         <v>6</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:6" ht="15">
       <c r="A22" s="2"/>
-      <c r="B22" s="5" t="s">
+      <c r="B22" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D22" s="4" t="n">
+      <c r="C22" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D22" s="4">
         <v>7</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="n">
+    <row r="23" spans="1:6" ht="15">
+      <c r="A23" s="2">
         <v>8</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C23" s="4"/>
@@ -768,53 +782,53 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:6" ht="15">
       <c r="A24" s="2"/>
-      <c r="B24" s="5" t="s">
+      <c r="B24" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" s="4" t="n">
+      <c r="C24" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D24" s="4">
         <v>100</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:6" ht="15">
       <c r="A25" s="2"/>
-      <c r="B25" s="5" t="s">
+      <c r="B25" t="s" s="5">
         <v>11</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" s="4" t="n">
+      <c r="C25" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D25" s="4">
         <v>888</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:6" ht="15">
       <c r="A26" s="2"/>
-      <c r="B26" s="5" t="s">
+      <c r="B26" t="s" s="5">
         <v>12</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D26" s="4" t="n">
+      <c r="C26" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D26" s="4">
         <v>777</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="n">
+    <row r="27" spans="1:6" ht="15">
+      <c r="A27" s="2">
         <v>6</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" t="s" s="3">
         <v>8</v>
       </c>
       <c r="C27" s="4"/>
@@ -822,89 +836,89 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:6" ht="15">
       <c r="A28" s="2"/>
-      <c r="B28" s="5" t="s">
+      <c r="B28" t="s" s="5">
         <v>9</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" s="4" t="n">
+      <c r="C28" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D28" s="4">
         <v>100</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:6" ht="15">
       <c r="A29" s="2"/>
-      <c r="B29" s="5" t="s">
+      <c r="B29" t="s" s="5">
         <v>10</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D29" s="4" t="n">
+      <c r="C29" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D29" s="4">
         <v>100</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="1048522" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048523" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048524" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048525" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048526" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048527" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048528" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048529" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048530" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048531" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048532" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048533" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048534" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048535" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048536" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048537" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048538" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048539" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048540" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048541" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048542" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048543" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048544" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048545" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048546" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048547" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048548" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048549" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048550" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048551" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048552" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048553" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" ht="12.75"/>
+    <row r="1048523" ht="12.75"/>
+    <row r="1048524" ht="12.75"/>
+    <row r="1048525" ht="12.75"/>
+    <row r="1048526" ht="12.75"/>
+    <row r="1048527" ht="12.75"/>
+    <row r="1048528" ht="12.75"/>
+    <row r="1048529" ht="12.75"/>
+    <row r="1048530" ht="12.75"/>
+    <row r="1048531" ht="12.75"/>
+    <row r="1048532" ht="12.75"/>
+    <row r="1048533" ht="12.75"/>
+    <row r="1048534" ht="12.75"/>
+    <row r="1048535" ht="12.75"/>
+    <row r="1048536" ht="12.75"/>
+    <row r="1048537" ht="12.75"/>
+    <row r="1048538" ht="12.75"/>
+    <row r="1048539" ht="12.75"/>
+    <row r="1048540" ht="12.75"/>
+    <row r="1048541" ht="12.75"/>
+    <row r="1048542" ht="12.75"/>
+    <row r="1048543" ht="12.75"/>
+    <row r="1048544" ht="12.75"/>
+    <row r="1048545" ht="12.75"/>
+    <row r="1048546" ht="12.75"/>
+    <row r="1048547" ht="12.75"/>
+    <row r="1048548" ht="12.75"/>
+    <row r="1048549" ht="12.75"/>
+    <row r="1048550" ht="12.75"/>
+    <row r="1048551" ht="12.75"/>
+    <row r="1048552" ht="12.75"/>
+    <row r="1048553" ht="12.75"/>
+    <row r="1048554" ht="12.75"/>
+    <row r="1048555" ht="12.75"/>
+    <row r="1048556" ht="12.75"/>
+    <row r="1048557" ht="12.75"/>
+    <row r="1048558" ht="12.75"/>
+    <row r="1048559" ht="12.75"/>
+    <row r="1048560" ht="12.75"/>
+    <row r="1048561" ht="12.75"/>
+    <row r="1048562" ht="12.75"/>
+    <row r="1048563" ht="12.75"/>
+    <row r="1048564" ht="12.75"/>
+    <row r="1048565" ht="12.75"/>
+    <row r="1048566" ht="12.75"/>
+    <row r="1048567" ht="12.75"/>
+    <row r="1048568" ht="12.75"/>
+    <row r="1048569" ht="12.75"/>
+    <row r="1048570" ht="12.75"/>
+    <row r="1048571" ht="12.75"/>
+    <row r="1048572" ht="12.75"/>
+    <row r="1048573" ht="12.75"/>
+    <row r="1048574" ht="12.75"/>
+    <row r="1048575" ht="12.75"/>
+    <row r="1048576" ht="12.75"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:A2"/>
@@ -917,12 +931,332 @@
     <mergeCell ref="A23:A26"/>
     <mergeCell ref="A27:A29"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <phoneticPr fontId="1"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" scale="100" orientation="portrait" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr/>
+  <cols>
+    <col min="1" max="1" width="10.14" customWidth="1"/>
+    <col min="2" max="2" width="38.47" customWidth="1"/>
+    <col min="3" max="3" width="10.7" customWidth="1"/>
+    <col min="4" max="4" width="7.86" customWidth="1"/>
+    <col min="5" max="5" width="7.35" customWidth="1"/>
+    <col min="6" max="6" width="7.84" customWidth="1"/>
+    <col min="7" max="9" width="9.14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15" customHeight="1">
+      <c r="A1" s="2">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s" s="3">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1">
+      <c r="A2" s="2"/>
+      <c r="B2" t="s" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
+        <v>200</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1">
+      <c r="A3" s="2"/>
+      <c r="B3" t="s" s="5">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4">
+        <v>999</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1">
+      <c r="A4" s="2"/>
+      <c r="B4" t="s" s="5">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
+        <v>888</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1">
+      <c r="A5" s="2"/>
+      <c r="B5" t="s" s="5">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
+        <v>777</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:9" ht="15" customHeight="1">
+      <c r="A6" s="2">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s" s="3">
+        <v>3</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" ht="15" customHeight="1">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s" s="5">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D7" s="4">
+        <v>207</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1">
+      <c r="A8" s="2"/>
+      <c r="B8" t="s" s="5">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
+        <v>206</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1">
+      <c r="A9" s="2"/>
+      <c r="B9" t="s" s="5">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4">
+        <v>205</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="15" customHeight="1">
+      <c r="A10" s="2">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s" s="3">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1">
+      <c r="A11" s="2"/>
+      <c r="B11" t="s" s="5">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
+        <v>100</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1">
+      <c r="A12" s="2"/>
+      <c r="B12" t="s" s="5">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
+        <v>999</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" ht="15" customHeight="1">
+      <c r="A13" s="2"/>
+      <c r="B13" t="s" s="5">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D13" s="4">
+        <v>888</v>
+      </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="15" customHeight="1">
+      <c r="A14" s="2"/>
+      <c r="B14" t="s" s="5">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4">
+        <v>777</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:9" ht="15" customHeight="1">
+      <c r="A15" s="2">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s" s="3">
+        <v>8</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:9" ht="15" customHeight="1">
+      <c r="A16" s="2"/>
+      <c r="B16" t="s" s="5">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D16" s="4">
+        <v>200</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" ht="15" customHeight="1">
+      <c r="A17" s="2"/>
+      <c r="B17" t="s" s="5">
+        <v>10</v>
+      </c>
+      <c r="C17" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D17" s="4">
+        <v>200</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18" spans="1:6" ht="15" customHeight="1">
+      <c r="A18" s="2">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s" s="3">
+        <v>0</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+    </row>
+    <row r="19" spans="1:6" ht="15" customHeight="1">
+      <c r="A19" s="2"/>
+      <c r="B19" t="s" s="5">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D19" s="4">
+        <v>100</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20" spans="1:6" ht="15" customHeight="1">
+      <c r="A20" s="2"/>
+      <c r="B20" t="s" s="5">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4">
+        <v>888</v>
+      </c>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:6" ht="15" customHeight="1">
+      <c r="A21" s="2"/>
+      <c r="B21" t="s" s="5">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4">
+        <v>777</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A21"/>
+  </mergeCells>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
merged-cells-ext: Correct accumulation of grouped entries with different order and size.
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Range_Merged.xlsx
+++ b/Ref_Files/Test_Range_Merged.xlsx
@@ -719,7 +719,7 @@
         <v>2</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -737,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -751,7 +751,7 @@
         <v>2</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>

</xml_diff>

<commit_message>
merged-cells-ext: fixed compilation warnings
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Range_Merged.xlsx
+++ b/Ref_Files/Test_Range_Merged.xlsx
@@ -1,34 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr filterPrivacy="1"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView activeTab="0" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="КСС_ОП1" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="Prices" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">#REF!</definedName>
+    <definedName name="_Hlk165973344" localSheetId="0" hidden="0">#REF!</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="13">
-  <si>
-    <t xml:space="preserve">Операция Х-00100, с два реда</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="13">
+  <si>
+    <t>Операция Х-00100, с два реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00100 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <r>
@@ -39,7 +37,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">m</t>
+      <t>m</t>
     </r>
     <r>
       <rPr>
@@ -50,48 +48,59 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">3</t>
+      <t>3</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00200, с четири реда</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00200, с четири реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00201 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00202 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00203 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-99999 измерване</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00300, с три реда</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00300, с три реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00301 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00302 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-88888 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-77777 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,14 +148,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
@@ -155,58 +164,58 @@
     </border>
   </borders>
   <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -217,11 +226,17 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Тема на Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема на Office">
   <a:themeElements>
     <a:clrScheme name="Оffice">
       <a:dk1>
@@ -263,12 +278,12 @@
     </a:clrScheme>
     <a:fontScheme name="Оffice">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -300,7 +315,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -324,7 +339,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -384,38 +399,37 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:XFD29"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" outlineLevelCol="0" outlineLevelRow="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.84"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="7" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16365" min="14" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16366" style="1" width="10.16"/>
+    <col min="1" max="1" width="10.14" customWidth="1" style="1"/>
+    <col min="2" max="2" width="38.47" customWidth="1" style="1"/>
+    <col min="3" max="3" width="10.7" customWidth="1" style="1"/>
+    <col min="4" max="4" width="7.86" customWidth="1" style="1"/>
+    <col min="5" max="5" width="7.35" customWidth="1" style="1"/>
+    <col min="6" max="6" width="7.84" customWidth="1" style="1"/>
+    <col min="7" max="10" width="9.14" customWidth="1" style="1"/>
+    <col min="14" max="16365" width="9.14" customWidth="1" style="1"/>
+    <col min="16366" max="16384" width="10.16" customWidth="1" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="n">
+    <row r="1" spans="1:6" ht="15">
+      <c r="A1" s="2">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C1" s="4"/>
@@ -423,25 +437,25 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:6" ht="15">
       <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4" t="n">
+      <c r="C2" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
         <v>100</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
     </row>
-    <row r="3" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="3" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C3" s="4"/>
@@ -453,15 +467,15 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A4" s="2"/>
-      <c r="B4" s="5" t="s">
+      <c r="B4" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="C4" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
         <v>100</v>
       </c>
       <c r="E4" s="4"/>
@@ -471,39 +485,39 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:6" ht="15">
       <c r="A5" s="2"/>
-      <c r="B5" s="5" t="s">
+      <c r="B5" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="C5" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
         <v>100</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:6" ht="15">
       <c r="A6" s="2"/>
-      <c r="B6" s="5" t="s">
+      <c r="B6" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="C6" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4">
         <v>100</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+    <row r="7" spans="1:6" ht="15">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C7" s="4"/>
@@ -511,25 +525,25 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:6" ht="15">
       <c r="A8" s="2"/>
-      <c r="B8" s="5" t="s">
+      <c r="B8" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="C8" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
         <v>100</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+    <row r="9" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A9" s="2">
         <v>4</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C9" s="4"/>
@@ -541,15 +555,15 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
+      <c r="B10" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="C10" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D10" s="4">
         <v>100</v>
       </c>
       <c r="E10" s="4"/>
@@ -559,39 +573,39 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:6" ht="15">
       <c r="A11" s="2"/>
-      <c r="B11" s="5" t="s">
+      <c r="B11" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="4" t="n">
+      <c r="C11" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
         <v>100</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:6" ht="15">
       <c r="A12" s="2"/>
-      <c r="B12" s="5" t="s">
+      <c r="B12" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D12" s="4" t="n">
+      <c r="C12" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
         <v>100</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+    <row r="13" spans="1:6" ht="15">
+      <c r="A13" s="2">
         <v>5</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C13" s="4"/>
@@ -599,39 +613,39 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:6" ht="15">
       <c r="A14" s="2"/>
-      <c r="B14" s="5" t="s">
+      <c r="B14" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="4" t="n">
+      <c r="C14" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4">
         <v>100</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:6" ht="15">
       <c r="A15" s="2"/>
-      <c r="B15" s="5" t="s">
+      <c r="B15" t="s" s="5">
         <v>7</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D15" s="4" t="n">
+      <c r="C15" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4">
         <v>999</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
+    <row r="16" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A16" s="2">
         <v>6</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" t="s" s="3">
         <v>8</v>
       </c>
       <c r="C16" s="4"/>
@@ -643,15 +657,15 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A17" s="2"/>
-      <c r="B17" s="5" t="s">
+      <c r="B17" t="s" s="5">
         <v>9</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D17" s="4" t="n">
+      <c r="C17" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D17" s="4">
         <v>100</v>
       </c>
       <c r="E17" s="4"/>
@@ -661,15 +675,15 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:16384" ht="15">
       <c r="A18" s="2"/>
-      <c r="B18" s="5" t="s">
+      <c r="B18" t="s" s="5">
         <v>10</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="4" t="n">
+      <c r="C18" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D18" s="4">
         <v>100</v>
       </c>
       <c r="E18" s="4"/>
@@ -694,11 +708,11 @@
       <c r="XFC18" s="6"/>
       <c r="XFD18" s="6"/>
     </row>
-    <row r="19" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="n">
+    <row r="19" spans="1:10" ht="15" customFormat="1" s="6">
+      <c r="A19" s="2">
         <v>7</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" t="s" s="3">
         <v>3</v>
       </c>
       <c r="C19" s="4"/>
@@ -710,15 +724,15 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" s="6" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:10" ht="15" customFormat="1" s="6">
       <c r="A20" s="2"/>
-      <c r="B20" s="5" t="s">
+      <c r="B20" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="4" t="n">
+      <c r="C20" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4">
         <v>3</v>
       </c>
       <c r="E20" s="4"/>
@@ -728,39 +742,39 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:6" ht="15">
       <c r="A21" s="2"/>
-      <c r="B21" s="5" t="s">
+      <c r="B21" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" s="4" t="n">
+      <c r="C21" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4">
         <v>2</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:6" ht="15">
       <c r="A22" s="2"/>
-      <c r="B22" s="5" t="s">
+      <c r="B22" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D22" s="4" t="n">
+      <c r="C22" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D22" s="4">
         <v>1</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="n">
+    <row r="23" spans="1:6" ht="15">
+      <c r="A23" s="2">
         <v>8</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" t="s" s="3">
         <v>0</v>
       </c>
       <c r="C23" s="4"/>
@@ -768,53 +782,53 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:6" ht="15">
       <c r="A24" s="2"/>
-      <c r="B24" s="5" t="s">
+      <c r="B24" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" s="4" t="n">
+      <c r="C24" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D24" s="4">
         <v>100</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:6" ht="15">
       <c r="A25" s="2"/>
-      <c r="B25" s="5" t="s">
+      <c r="B25" t="s" s="5">
         <v>11</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" s="4" t="n">
+      <c r="C25" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D25" s="4">
         <v>888</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:6" ht="15">
       <c r="A26" s="2"/>
-      <c r="B26" s="5" t="s">
+      <c r="B26" t="s" s="5">
         <v>12</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D26" s="4" t="n">
+      <c r="C26" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D26" s="4">
         <v>777</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="n">
+    <row r="27" spans="1:6" ht="15">
+      <c r="A27" s="2">
         <v>6</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" t="s" s="3">
         <v>8</v>
       </c>
       <c r="C27" s="4"/>
@@ -822,89 +836,89 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:6" ht="15">
       <c r="A28" s="2"/>
-      <c r="B28" s="5" t="s">
+      <c r="B28" t="s" s="5">
         <v>9</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" s="4" t="n">
+      <c r="C28" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D28" s="4">
         <v>100</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:6" ht="15">
       <c r="A29" s="2"/>
-      <c r="B29" s="5" t="s">
+      <c r="B29" t="s" s="5">
         <v>10</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D29" s="4" t="n">
+      <c r="C29" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D29" s="4">
         <v>100</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="1048522" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048523" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048524" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048525" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048526" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048527" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048528" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048529" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048530" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048531" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048532" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048533" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048534" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048535" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048536" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048537" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048538" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048539" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048540" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048541" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048542" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048543" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048544" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048545" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048546" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048547" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048548" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048549" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048550" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048551" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048552" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048553" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048522" ht="12.75"/>
+    <row r="1048523" ht="12.75"/>
+    <row r="1048524" ht="12.75"/>
+    <row r="1048525" ht="12.75"/>
+    <row r="1048526" ht="12.75"/>
+    <row r="1048527" ht="12.75"/>
+    <row r="1048528" ht="12.75"/>
+    <row r="1048529" ht="12.75"/>
+    <row r="1048530" ht="12.75"/>
+    <row r="1048531" ht="12.75"/>
+    <row r="1048532" ht="12.75"/>
+    <row r="1048533" ht="12.75"/>
+    <row r="1048534" ht="12.75"/>
+    <row r="1048535" ht="12.75"/>
+    <row r="1048536" ht="12.75"/>
+    <row r="1048537" ht="12.75"/>
+    <row r="1048538" ht="12.75"/>
+    <row r="1048539" ht="12.75"/>
+    <row r="1048540" ht="12.75"/>
+    <row r="1048541" ht="12.75"/>
+    <row r="1048542" ht="12.75"/>
+    <row r="1048543" ht="12.75"/>
+    <row r="1048544" ht="12.75"/>
+    <row r="1048545" ht="12.75"/>
+    <row r="1048546" ht="12.75"/>
+    <row r="1048547" ht="12.75"/>
+    <row r="1048548" ht="12.75"/>
+    <row r="1048549" ht="12.75"/>
+    <row r="1048550" ht="12.75"/>
+    <row r="1048551" ht="12.75"/>
+    <row r="1048552" ht="12.75"/>
+    <row r="1048553" ht="12.75"/>
+    <row r="1048554" ht="12.75"/>
+    <row r="1048555" ht="12.75"/>
+    <row r="1048556" ht="12.75"/>
+    <row r="1048557" ht="12.75"/>
+    <row r="1048558" ht="12.75"/>
+    <row r="1048559" ht="12.75"/>
+    <row r="1048560" ht="12.75"/>
+    <row r="1048561" ht="12.75"/>
+    <row r="1048562" ht="12.75"/>
+    <row r="1048563" ht="12.75"/>
+    <row r="1048564" ht="12.75"/>
+    <row r="1048565" ht="12.75"/>
+    <row r="1048566" ht="12.75"/>
+    <row r="1048567" ht="12.75"/>
+    <row r="1048568" ht="12.75"/>
+    <row r="1048569" ht="12.75"/>
+    <row r="1048570" ht="12.75"/>
+    <row r="1048571" ht="12.75"/>
+    <row r="1048572" ht="12.75"/>
+    <row r="1048573" ht="12.75"/>
+    <row r="1048574" ht="12.75"/>
+    <row r="1048575" ht="12.75"/>
+    <row r="1048576" ht="12.75"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:A2"/>
@@ -917,12 +931,208 @@
     <mergeCell ref="A23:A26"/>
     <mergeCell ref="A27:A29"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <phoneticPr fontId="1"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" scale="100" orientation="portrait" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr/>
+  <cols>
+    <col min="1" max="1" width="10.14" customWidth="1"/>
+    <col min="2" max="2" width="38.47" customWidth="1"/>
+    <col min="3" max="3" width="10.7" customWidth="1"/>
+    <col min="4" max="4" width="7.86" customWidth="1"/>
+    <col min="5" max="5" width="7.35" customWidth="1"/>
+    <col min="6" max="6" width="7.84" customWidth="1"/>
+    <col min="7" max="9" width="9.14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="15" customHeight="1">
+      <c r="A1" s="2">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="3">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1">
+      <c r="A2" s="2"/>
+      <c r="B2" t="s" s="5">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
+        <v>400</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1">
+      <c r="A3" s="2"/>
+      <c r="B3" t="s" s="5">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4">
+        <v>999</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1">
+      <c r="A4" s="2"/>
+      <c r="B4" t="s" s="5">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
+        <v>888</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1">
+      <c r="A5" s="2"/>
+      <c r="B5" t="s" s="5">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
+        <v>777</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:9" ht="15" customHeight="1">
+      <c r="A6" s="2">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s" s="3">
+        <v>3</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" ht="15" customHeight="1">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s" s="5">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D7" s="4">
+        <v>201</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1">
+      <c r="A8" s="2"/>
+      <c r="B8" t="s" s="5">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
+        <v>202</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1">
+      <c r="A9" s="2"/>
+      <c r="B9" t="s" s="5">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4">
+        <v>203</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" ht="15" customHeight="1">
+      <c r="A10" s="2">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s" s="3">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" ht="15" customHeight="1">
+      <c r="A11" s="2"/>
+      <c r="B11" t="s" s="5">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
+        <v>200</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1">
+      <c r="A12" s="2"/>
+      <c r="B12" t="s" s="5">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
+        <v>200</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A12"/>
+  </mergeCells>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>
 </file>
</xml_diff>